<commit_message>
Memperbaiki fitur penginputan form input pengisian
</commit_message>
<xml_diff>
--- a/snd2.xlsx
+++ b/snd2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josua\Downloads\Magang_Pertamina\Project Autofill RSD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73E2223C-309B-4E1F-886E-01AF2C0F797C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69E0E32F-F254-4616-B010-93ED18FFF86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3072" yWindow="3072" windowWidth="17280" windowHeight="9960" xr2:uid="{9A2200E5-FF86-4C93-BFF4-5ACC1DA43524}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9A2200E5-FF86-4C93-BFF4-5ACC1DA43524}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Tanggal Shipment</t>
   </si>
@@ -66,9 +66,6 @@
     <t>ALFREY ROMPAH [73100236/905]</t>
   </si>
   <si>
-    <t>8142204097,8142201374,8142204098,</t>
-  </si>
-  <si>
     <t>1660959,1660960,1660961,1660962,1660963,1660964,</t>
   </si>
   <si>
@@ -100,6 +97,9 @@
   </si>
   <si>
     <t>B9686SXXX</t>
+  </si>
+  <si>
+    <t>BIOSOLAR B50;</t>
   </si>
 </sst>
 </file>
@@ -135,10 +135,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="47" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -500,22 +503,22 @@
         <v>46237.681788888891</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
         <v>9</v>
       </c>
       <c r="E2">
-        <v>24</v>
-      </c>
-      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="3">
+        <v>8142204097</v>
+      </c>
+      <c r="G2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" t="s">
         <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -526,22 +529,22 @@
         <v>46237.654189814813</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E3">
         <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G3" t="s">
         <v>8</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -552,22 +555,22 @@
         <v>46237.28125</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E4">
         <v>24</v>
       </c>
       <c r="F4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" t="s">
         <v>18</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>19</v>
-      </c>
-      <c r="H4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Memperbaiki input meter awal dan akhir pada modal pengisian
</commit_message>
<xml_diff>
--- a/snd2.xlsx
+++ b/snd2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josua\Downloads\Magang_Pertamina\Project Autofill RSD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69E0E32F-F254-4616-B010-93ED18FFF86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1725D0F6-E588-4359-A427-5E28EB7093DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9A2200E5-FF86-4C93-BFF4-5ACC1DA43524}"/>
   </bookViews>
@@ -60,9 +60,6 @@
     <t>Segel</t>
   </si>
   <si>
-    <t>PERTALITE;</t>
-  </si>
-  <si>
     <t>ALFREY ROMPAH [73100236/905]</t>
   </si>
   <si>
@@ -100,6 +97,9 @@
   </si>
   <si>
     <t>BIOSOLAR B50;</t>
+  </si>
+  <si>
+    <t>PERTALITE;BIOSOLAR B50;</t>
   </si>
 </sst>
 </file>
@@ -503,10 +503,10 @@
         <v>46237.681788888891</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E2">
         <v>8</v>
@@ -515,10 +515,10 @@
         <v>8142204097</v>
       </c>
       <c r="G2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -529,22 +529,22 @@
         <v>46237.654189814813</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E3">
         <v>16</v>
       </c>
       <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
         <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -555,22 +555,22 @@
         <v>46237.28125</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E4">
         <v>24</v>
       </c>
       <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" t="s">
         <v>17</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>18</v>
-      </c>
-      <c r="H4" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Perbaikan Bug saat pembukaan link Nomor penyaluran agar tidak looping menggunakan DOM Attribute Lock
</commit_message>
<xml_diff>
--- a/snd2.xlsx
+++ b/snd2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Josua\Downloads\Magang_Pertamina\Project Autofill RSD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1725D0F6-E588-4359-A427-5E28EB7093DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD00EC43-DFF8-437C-AFD1-49A565BB7357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{9A2200E5-FF86-4C93-BFF4-5ACC1DA43524}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{9A2200E5-FF86-4C93-BFF4-5ACC1DA43524}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Tanggal Shipment</t>
   </si>
@@ -60,12 +60,6 @@
     <t>Segel</t>
   </si>
   <si>
-    <t>ALFREY ROMPAH [73100236/905]</t>
-  </si>
-  <si>
-    <t>1660959,1660960,1660961,1660962,1660963,1660964,</t>
-  </si>
-  <si>
     <t>Marcelino Mardiani Kalengkongan [73116590/1181]</t>
   </si>
   <si>
@@ -75,9 +69,6 @@
     <t>1660951,1660952,1660953,1660954,</t>
   </si>
   <si>
-    <t>DB8016XXX</t>
-  </si>
-  <si>
     <t>B9726SXXX</t>
   </si>
   <si>
@@ -94,9 +85,6 @@
   </si>
   <si>
     <t>B9686SXXX</t>
-  </si>
-  <si>
-    <t>BIOSOLAR B50;</t>
   </si>
   <si>
     <t>PERTALITE;BIOSOLAR B50;</t>
@@ -496,30 +484,9 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
-        <v>46237.632488425923</v>
-      </c>
-      <c r="B2" s="2">
-        <v>46237.681788888891</v>
-      </c>
-      <c r="C2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2">
-        <v>8</v>
-      </c>
-      <c r="F2" s="3">
-        <v>8142204097</v>
-      </c>
-      <c r="G2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H2" t="s">
-        <v>9</v>
-      </c>
+      <c r="A2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
@@ -529,22 +496,22 @@
         <v>46237.654189814813</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E3">
         <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="H3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -555,22 +522,22 @@
         <v>46237.28125</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E4">
         <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="H4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>